<commit_message>
fixed an issue in the menu_items table that included combos in course 1 (now course 4)
</commit_message>
<xml_diff>
--- a/scripts/menu.xlsx
+++ b/scripts/menu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loren\Desktop\Simulation\Progetto\Restaurant_2025\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1EE37F2-34E0-4D3D-AC17-7B7EC89036CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C8E2BE-33E5-4DFE-856D-D9C90D13C2CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14310" yWindow="0" windowWidth="14580" windowHeight="19290" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="19420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="menu_items" sheetId="2" r:id="rId1"/>
@@ -22,16 +22,10 @@
   </sheets>
   <definedNames>
     <definedName name="DatiEsterni_1" localSheetId="0" hidden="1">menu_items!$A$1:$P$33</definedName>
-    <definedName name="DatiEsterni_1" localSheetId="0" hidden="1">menu_items!$A$1:$P$33</definedName>
-    <definedName name="DatiEsterni_2" localSheetId="4" hidden="1">copula_lunch_correlation!$A$1:$G$7</definedName>
     <definedName name="DatiEsterni_2" localSheetId="4" hidden="1">copula_lunch_correlation!$A$1:$G$7</definedName>
     <definedName name="DatiEsterni_2" localSheetId="1" hidden="1">copula_menu_marginals!$A$1:$C$18</definedName>
-    <definedName name="DatiEsterni_2" localSheetId="1" hidden="1">copula_menu_marginals!$A$1:$C$18</definedName>
-    <definedName name="DatiEsterni_3" localSheetId="3" hidden="1">'copula_break_correlation'!$A$1:$C$3</definedName>
     <definedName name="DatiEsterni_3" localSheetId="3" hidden="1">'copula_break_correlation'!$A$1:$C$3</definedName>
     <definedName name="DatiEsterni_3" localSheetId="5" hidden="1">copula_dinner_correlation!$A$1:$G$7</definedName>
-    <definedName name="DatiEsterni_3" localSheetId="5" hidden="1">copula_dinner_correlation!$A$1:$G$7</definedName>
-    <definedName name="DatiEsterni_4" localSheetId="2" hidden="1">'copula_breakfast_correlation'!$A$1:$D$4</definedName>
     <definedName name="DatiEsterni_4" localSheetId="2" hidden="1">'copula_breakfast_correlation'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -467,16 +461,16 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D8B0271-1D61-41BA-BC5B-F689FABB7AB6}" name="menu_items" displayName="menu_items" ref="A1:P33" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:P33" xr:uid="{E72E3C1B-3A6E-4772-96C0-B78989E87280}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{00A19D1C-D261-471D-B81D-3B09AAB118BD}" uniqueName="1" name="name" queryTableFieldId="1" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{206D0B97-AF7C-42DE-8089-C23290EBD056}" uniqueName="2" name="dayPart" queryTableFieldId="2" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{2E037A64-0660-451E-B72A-1C871D5F10D8}" uniqueName="3" name="category" queryTableFieldId="3" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{00A19D1C-D261-471D-B81D-3B09AAB118BD}" uniqueName="1" name="name" queryTableFieldId="1" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{206D0B97-AF7C-42DE-8089-C23290EBD056}" uniqueName="2" name="dayPart" queryTableFieldId="2" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{2E037A64-0660-451E-B72A-1C871D5F10D8}" uniqueName="3" name="category" queryTableFieldId="3" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{969F2254-CB09-476C-A99D-5AB38A62CD4E}" uniqueName="4" name="course" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{C6F7F582-1F26-4016-91AD-4F12D8E5EAF6}" uniqueName="5" name="popularityWeight" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{862ABBE4-D89E-4E1B-BA8C-D0C68C7F1430}" uniqueName="6" name="price" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{06559A55-CEC0-4333-91A4-D7FD4836EADD}" uniqueName="7" name="prepTimeMeanMin" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{7B9473CB-9E61-42AB-A2F4-A2FECF5663D4}" uniqueName="8" name="prepTimeSdMin" queryTableFieldId="8"/>
     <tableColumn id="9" xr3:uid="{B0096415-69DE-49A7-9BF7-61B97368A6D2}" uniqueName="9" name="complexity" queryTableFieldId="9"/>
-    <tableColumn id="10" xr3:uid="{F8F425FE-F4DF-4689-93B9-9E6F33BE921F}" uniqueName="10" name="kitchenStation" queryTableFieldId="10" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{F8F425FE-F4DF-4689-93B9-9E6F33BE921F}" uniqueName="10" name="kitchenStation" queryTableFieldId="10" dataDxfId="5"/>
     <tableColumn id="11" xr3:uid="{4BCE7A2D-659F-424F-8521-C2523BF681E3}" uniqueName="11" name="requiresKitchen" queryTableFieldId="11"/>
     <tableColumn id="12" xr3:uid="{A36CA02C-373F-4884-9AB3-CBEF99923C7A}" uniqueName="12" name="isCombo" queryTableFieldId="12"/>
     <tableColumn id="13" xr3:uid="{3BF4BCCD-4385-4E5D-B5F1-492BF92716C6}" uniqueName="13" name="isFixedMenu" queryTableFieldId="13"/>
@@ -492,8 +486,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FC8E48F-6A69-453C-99ED-E875FCDB7425}" name="copula_marginals" displayName="copula_marginals" ref="A1:D18" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D18" xr:uid="{E9512F47-E937-443E-9B1F-BE61055B98E4}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D0659F2D-8BAB-42E6-9B39-F0A8FBF58867}" uniqueName="1" name="dayPart" queryTableFieldId="1" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{112A78DA-0E67-4465-9CA6-710D9BEECE37}" uniqueName="2" name="variable" queryTableFieldId="2" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{D0659F2D-8BAB-42E6-9B39-F0A8FBF58867}" uniqueName="1" name="dayPart" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{112A78DA-0E67-4465-9CA6-710D9BEECE37}" uniqueName="2" name="variable" queryTableFieldId="2" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{8D15E6A7-35AE-4B65-820F-91CFCE1286F9}" uniqueName="3" name="marginal_probability" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{8BF211C3-E2A0-43BC-A80E-C63CF9D29C7D}" uniqueName="4" name="position" queryTableFieldId="4"/>
   </tableColumns>
@@ -505,7 +499,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{86F8DF43-4949-43DD-B190-ECA1A8184BB1}" name="copula_breakfast_correlation" displayName="copula_breakfast_correlation" ref="A1:D4" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D4" xr:uid="{BE7DE44D-2DBC-4260-B1A0-DD0022E7EF5E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D405A4A4-3D72-49AA-9B0D-58EA4DDA3930}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{D405A4A4-3D72-49AA-9B0D-58EA4DDA3930}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{9B6705B6-582C-4D3B-9589-D71017366FDB}" uniqueName="2" name="main" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{384654C0-BDC2-4EF5-BE2A-71B8D21EC7BC}" uniqueName="3" name="drink" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{A8923EDE-5B2B-44E5-9EE2-C06F837CF20E}" uniqueName="4" name="combo" queryTableFieldId="4"/>
@@ -518,7 +512,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7ECD888C-2804-4A3A-825D-2A98174492A1}" name="copula_break_correlation" displayName="copula_break_correlation" ref="A1:C3" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C3" xr:uid="{E1DB2A7D-214B-4EDA-93BE-7944E1899C7B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{D6D6812D-CCD7-454F-83E2-41742110D9E8}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D6D6812D-CCD7-454F-83E2-41742110D9E8}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{685C995E-5E2F-44FF-82DF-AD4FF1FB9AFF}" uniqueName="2" name="main" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{C5FD3759-004D-4A34-B6BF-77519F37E5BB}" uniqueName="3" name="drink" queryTableFieldId="3"/>
   </tableColumns>
@@ -530,7 +524,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{53168AE0-663A-44CC-B480-A8986D8FD424}" name="copula_lunch_correlation__2" displayName="copula_lunch_correlation__2" ref="A1:G7" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G7" xr:uid="{43E3CE34-FCB7-466B-8B5D-B62B78A22057}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1D6EC97C-FE66-4EE0-B3AD-FE4DCE26CCAF}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{1D6EC97C-FE66-4EE0-B3AD-FE4DCE26CCAF}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{DEA1F054-4624-4A1B-8CB8-8F1A08557B0D}" uniqueName="2" name="fixed_menu" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{C4ECF60B-8C0C-4D2D-99F2-14D2A254D5B9}" uniqueName="3" name="course1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{9395D41D-545A-4A77-B907-0885B99E04EB}" uniqueName="4" name="course2" queryTableFieldId="4"/>
@@ -546,7 +540,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A6191000-A3D2-43E4-89CA-07E6937A7F0A}" name="copula_dinner_correlation__2" displayName="copula_dinner_correlation__2" ref="A1:G7" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G7" xr:uid="{3EB7145D-72D8-42E0-ABCA-09A7559072D3}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{E9E1F63E-5651-4BC3-94C3-5D2B86D76CA0}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{E9E1F63E-5651-4BC3-94C3-5D2B86D76CA0}" uniqueName="1" name="variable" queryTableFieldId="1" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{1595AA1C-4819-46C8-A476-9B29B57AE3D6}" uniqueName="2" name="fixed_menu" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{2FCC3078-A1E8-44CE-A421-EAEE298710D4}" uniqueName="3" name="course1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{A9C512FF-273B-49E6-99A8-0A0ABF11B61F}" uniqueName="4" name="course2" queryTableFieldId="4"/>
@@ -1203,7 +1197,7 @@
         <v>37</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E8">
         <v>18</v>
@@ -2053,7 +2047,7 @@
         <v>1</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E25">
         <v>22</v>
@@ -2453,7 +2447,7 @@
         <v>1</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E33">
         <v>6</v>

</xml_diff>

<commit_message>
removed useless properties from the menu
</commit_message>
<xml_diff>
--- a/scripts/menu.xlsx
+++ b/scripts/menu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loren\Desktop\Simulation\Progetto\Restaurant_2025\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1840F6A-4BF8-4FA6-A519-4DA9CCBD564A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220B2D3E-7FB9-4577-B916-294558464776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="19420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="copula_dinner_correlation" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="DatiEsterni_1" localSheetId="0" hidden="1">menu_items!$A$1:$P$33</definedName>
+    <definedName name="DatiEsterni_1" localSheetId="0" hidden="1">menu_items!$A$1:$I$33</definedName>
     <definedName name="DatiEsterni_2" localSheetId="4" hidden="1">copula_lunch_correlation!$A$1:$G$7</definedName>
     <definedName name="DatiEsterni_2" localSheetId="1" hidden="1">copula_menu_marginals!$A$1:$C$18</definedName>
     <definedName name="DatiEsterni_3" localSheetId="3" hidden="1">'copula_break_correlation'!$A$1:$C$3</definedName>
@@ -61,10 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="72">
-  <si>
-    <t>HOT</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="62">
   <si>
     <t>FIXED_MENU</t>
   </si>
@@ -75,9 +72,6 @@
     <t>Full dinner menu</t>
   </si>
   <si>
-    <t>BAR</t>
-  </si>
-  <si>
     <t>DRINK</t>
   </si>
   <si>
@@ -87,9 +81,6 @@
     <t>Medium beer</t>
   </si>
   <si>
-    <t>COLD</t>
-  </si>
-  <si>
     <t>DESSERT</t>
   </si>
   <si>
@@ -199,27 +190,6 @@
   </si>
   <si>
     <t>available</t>
-  </si>
-  <si>
-    <t>eatingTimeMeanMin</t>
-  </si>
-  <si>
-    <t>serviceTimeMeanMin</t>
-  </si>
-  <si>
-    <t>isFixedMenu</t>
-  </si>
-  <si>
-    <t>isCombo</t>
-  </si>
-  <si>
-    <t>requiresKitchen</t>
-  </si>
-  <si>
-    <t>kitchenStation</t>
-  </si>
-  <si>
-    <t>complexity</t>
   </si>
   <si>
     <t>prepTimeSdMin</t>
@@ -318,10 +288,7 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -365,7 +332,7 @@
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatiEsterni_1" connectionId="6" xr16:uid="{13154D44-B857-400F-92BF-8B328A8E39D6}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="17">
-    <queryTableFields count="16">
+    <queryTableFields count="9">
       <queryTableField id="1" name="name" tableColumnId="1"/>
       <queryTableField id="2" name="dayPart" tableColumnId="2"/>
       <queryTableField id="3" name="category" tableColumnId="3"/>
@@ -374,15 +341,17 @@
       <queryTableField id="6" name="price" tableColumnId="6"/>
       <queryTableField id="7" name="prepTimeMeanMin" tableColumnId="7"/>
       <queryTableField id="8" name="prepTimeSdMin" tableColumnId="8"/>
-      <queryTableField id="9" name="complexity" tableColumnId="9"/>
-      <queryTableField id="10" name="kitchenStation" tableColumnId="10"/>
-      <queryTableField id="11" name="requiresKitchen" tableColumnId="11"/>
-      <queryTableField id="12" name="isCombo" tableColumnId="12"/>
-      <queryTableField id="13" name="isFixedMenu" tableColumnId="13"/>
-      <queryTableField id="14" name="serviceTimeMeanMin" tableColumnId="14"/>
-      <queryTableField id="15" name="eatingTimeMeanMin" tableColumnId="15"/>
       <queryTableField id="16" name="available" tableColumnId="16"/>
     </queryTableFields>
+    <queryTableDeletedFields count="7">
+      <deletedField name="complexity"/>
+      <deletedField name="kitchenStation"/>
+      <deletedField name="requiresKitchen"/>
+      <deletedField name="isCombo"/>
+      <deletedField name="isFixedMenu"/>
+      <deletedField name="serviceTimeMeanMin"/>
+      <deletedField name="eatingTimeMeanMin"/>
+    </queryTableDeletedFields>
   </queryTableRefresh>
 </queryTable>
 </file>
@@ -458,24 +427,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D8B0271-1D61-41BA-BC5B-F689FABB7AB6}" name="menu_items" displayName="menu_items" ref="A1:P33" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:P33" xr:uid="{E72E3C1B-3A6E-4772-96C0-B78989E87280}"/>
-  <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{00A19D1C-D261-471D-B81D-3B09AAB118BD}" uniqueName="1" name="name" queryTableFieldId="1" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{206D0B97-AF7C-42DE-8089-C23290EBD056}" uniqueName="2" name="dayPart" queryTableFieldId="2" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{2E037A64-0660-451E-B72A-1C871D5F10D8}" uniqueName="3" name="category" queryTableFieldId="3" dataDxfId="7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D8B0271-1D61-41BA-BC5B-F689FABB7AB6}" name="menu_items" displayName="menu_items" ref="A1:I33" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:I33" xr:uid="{E72E3C1B-3A6E-4772-96C0-B78989E87280}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{00A19D1C-D261-471D-B81D-3B09AAB118BD}" uniqueName="1" name="name" queryTableFieldId="1" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{206D0B97-AF7C-42DE-8089-C23290EBD056}" uniqueName="2" name="dayPart" queryTableFieldId="2" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{2E037A64-0660-451E-B72A-1C871D5F10D8}" uniqueName="3" name="category" queryTableFieldId="3" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{969F2254-CB09-476C-A99D-5AB38A62CD4E}" uniqueName="4" name="course" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{C6F7F582-1F26-4016-91AD-4F12D8E5EAF6}" uniqueName="5" name="popularityWeight" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{862ABBE4-D89E-4E1B-BA8C-D0C68C7F1430}" uniqueName="6" name="price" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{06559A55-CEC0-4333-91A4-D7FD4836EADD}" uniqueName="7" name="prepTimeMeanMin" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{7B9473CB-9E61-42AB-A2F4-A2FECF5663D4}" uniqueName="8" name="prepTimeSdMin" queryTableFieldId="8"/>
-    <tableColumn id="9" xr3:uid="{B0096415-69DE-49A7-9BF7-61B97368A6D2}" uniqueName="9" name="complexity" queryTableFieldId="9"/>
-    <tableColumn id="10" xr3:uid="{F8F425FE-F4DF-4689-93B9-9E6F33BE921F}" uniqueName="10" name="kitchenStation" queryTableFieldId="10" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{4BCE7A2D-659F-424F-8521-C2523BF681E3}" uniqueName="11" name="requiresKitchen" queryTableFieldId="11"/>
-    <tableColumn id="12" xr3:uid="{A36CA02C-373F-4884-9AB3-CBEF99923C7A}" uniqueName="12" name="isCombo" queryTableFieldId="12"/>
-    <tableColumn id="13" xr3:uid="{3BF4BCCD-4385-4E5D-B5F1-492BF92716C6}" uniqueName="13" name="isFixedMenu" queryTableFieldId="13"/>
-    <tableColumn id="14" xr3:uid="{8263480E-28C4-4D03-8FE7-80C59762CB0B}" uniqueName="14" name="serviceTimeMeanMin" queryTableFieldId="14"/>
-    <tableColumn id="15" xr3:uid="{C15F7CAA-B059-4B2D-A58A-8D5B56CEA1B5}" uniqueName="15" name="eatingTimeMeanMin" queryTableFieldId="15"/>
     <tableColumn id="16" xr3:uid="{A83CA9A1-F1E1-46F1-9F88-014C2CE1C136}" uniqueName="16" name="available" queryTableFieldId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -815,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D495744D-EC55-4DC0-B500-23BD333AC247}">
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.08984375" bestFit="1" customWidth="1"/>
@@ -836,65 +798,44 @@
     <col min="16" max="16" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="H1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L1" t="s">
-        <v>49</v>
-      </c>
-      <c r="M1" t="s">
-        <v>48</v>
-      </c>
-      <c r="N1" t="s">
-        <v>47</v>
-      </c>
-      <c r="O1" t="s">
-        <v>46</v>
-      </c>
-      <c r="P1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -911,40 +852,19 @@
       <c r="H2">
         <v>0.3</v>
       </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0.5</v>
-      </c>
-      <c r="O2">
-        <v>6</v>
-      </c>
-      <c r="P2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -961,40 +881,19 @@
       <c r="H3">
         <v>0.5</v>
       </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0.7</v>
-      </c>
-      <c r="O3">
-        <v>8</v>
-      </c>
-      <c r="P3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1011,40 +910,19 @@
       <c r="H4">
         <v>0.6</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K4" t="b">
-        <v>1</v>
-      </c>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0.6</v>
-      </c>
-      <c r="O4">
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
-      </c>
-      <c r="P4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1061,40 +939,19 @@
       <c r="H5">
         <v>0.2</v>
       </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0.4</v>
-      </c>
-      <c r="O5">
-        <v>7</v>
-      </c>
-      <c r="P5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1111,40 +968,19 @@
       <c r="H6">
         <v>0.3</v>
       </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6" t="s">
-        <v>4</v>
-      </c>
-      <c r="K6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M6" t="b">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0.5</v>
-      </c>
-      <c r="O6">
-        <v>8</v>
-      </c>
-      <c r="P6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1161,40 +997,19 @@
       <c r="H7">
         <v>1</v>
       </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7" t="s">
-        <v>4</v>
-      </c>
-      <c r="K7" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" t="b">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0.8</v>
-      </c>
-      <c r="O7">
-        <v>12</v>
-      </c>
-      <c r="P7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -1211,40 +1026,19 @@
       <c r="H8">
         <v>0.6</v>
       </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
-      <c r="J8" t="s">
-        <v>4</v>
-      </c>
-      <c r="K8" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" t="b">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>1</v>
-      </c>
-      <c r="O8">
-        <v>12</v>
-      </c>
-      <c r="P8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1261,40 +1055,19 @@
       <c r="H9">
         <v>0.2</v>
       </c>
-      <c r="I9">
-        <v>1</v>
-      </c>
-      <c r="J9" t="s">
-        <v>4</v>
-      </c>
-      <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" t="b">
-        <v>0</v>
-      </c>
-      <c r="M9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N9">
-        <v>0.4</v>
-      </c>
-      <c r="O9">
-        <v>6</v>
-      </c>
-      <c r="P9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1311,40 +1084,19 @@
       <c r="H10">
         <v>0.8</v>
       </c>
-      <c r="I10">
-        <v>1</v>
-      </c>
-      <c r="J10" t="s">
-        <v>4</v>
-      </c>
-      <c r="K10" t="b">
-        <v>1</v>
-      </c>
-      <c r="L10" t="b">
-        <v>0</v>
-      </c>
-      <c r="M10" t="b">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0.8</v>
-      </c>
-      <c r="O10">
-        <v>15</v>
-      </c>
-      <c r="P10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1361,40 +1113,19 @@
       <c r="H11">
         <v>0.7</v>
       </c>
-      <c r="I11">
-        <v>1</v>
-      </c>
-      <c r="J11" t="s">
-        <v>0</v>
-      </c>
-      <c r="K11" t="b">
-        <v>1</v>
-      </c>
-      <c r="L11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M11" t="b">
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <v>0.7</v>
-      </c>
-      <c r="O11">
-        <v>12</v>
-      </c>
-      <c r="P11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1411,40 +1142,19 @@
       <c r="H12">
         <v>0.8</v>
       </c>
-      <c r="I12">
-        <v>1</v>
-      </c>
-      <c r="J12" t="s">
-        <v>8</v>
-      </c>
-      <c r="K12" t="b">
-        <v>1</v>
-      </c>
-      <c r="L12" t="b">
-        <v>0</v>
-      </c>
-      <c r="M12" t="b">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>0.8</v>
-      </c>
-      <c r="O12">
-        <v>14</v>
-      </c>
-      <c r="P12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -1461,40 +1171,19 @@
       <c r="H13">
         <v>0.1</v>
       </c>
-      <c r="I13">
-        <v>1</v>
-      </c>
-      <c r="J13" t="s">
-        <v>4</v>
-      </c>
-      <c r="K13" t="b">
-        <v>0</v>
-      </c>
-      <c r="L13" t="b">
-        <v>0</v>
-      </c>
-      <c r="M13" t="b">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>0.3</v>
-      </c>
-      <c r="O13">
-        <v>8</v>
-      </c>
-      <c r="P13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -1511,40 +1200,19 @@
       <c r="H14">
         <v>0.3</v>
       </c>
-      <c r="I14">
-        <v>1</v>
-      </c>
-      <c r="J14" t="s">
-        <v>4</v>
-      </c>
-      <c r="K14" t="b">
-        <v>1</v>
-      </c>
-      <c r="L14" t="b">
-        <v>0</v>
-      </c>
-      <c r="M14" t="b">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0.5</v>
-      </c>
-      <c r="O14">
-        <v>6</v>
-      </c>
-      <c r="P14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -1561,40 +1229,19 @@
       <c r="H15">
         <v>0.5</v>
       </c>
-      <c r="I15">
-        <v>1</v>
-      </c>
-      <c r="J15" t="s">
-        <v>4</v>
-      </c>
-      <c r="K15" t="b">
-        <v>1</v>
-      </c>
-      <c r="L15" t="b">
-        <v>0</v>
-      </c>
-      <c r="M15" t="b">
-        <v>0</v>
-      </c>
-      <c r="N15">
-        <v>0.8</v>
-      </c>
-      <c r="O15">
-        <v>18</v>
-      </c>
-      <c r="P15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1611,40 +1258,19 @@
       <c r="H16">
         <v>1.5</v>
       </c>
-      <c r="I16">
-        <v>2</v>
-      </c>
-      <c r="J16" t="s">
-        <v>8</v>
-      </c>
-      <c r="K16" t="b">
-        <v>1</v>
-      </c>
-      <c r="L16" t="b">
-        <v>0</v>
-      </c>
-      <c r="M16" t="b">
-        <v>0</v>
-      </c>
-      <c r="N16">
-        <v>1</v>
-      </c>
-      <c r="O16">
-        <v>22</v>
-      </c>
-      <c r="P16" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1661,40 +1287,19 @@
       <c r="H17">
         <v>2</v>
       </c>
-      <c r="I17">
-        <v>2</v>
-      </c>
-      <c r="J17" t="s">
-        <v>0</v>
-      </c>
-      <c r="K17" t="b">
-        <v>1</v>
-      </c>
-      <c r="L17" t="b">
-        <v>0</v>
-      </c>
-      <c r="M17" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>1.2</v>
-      </c>
-      <c r="O17">
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>22</v>
       </c>
-      <c r="P17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>25</v>
-      </c>
       <c r="B18" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1711,40 +1316,19 @@
       <c r="H18">
         <v>2.5</v>
       </c>
-      <c r="I18">
-        <v>2</v>
-      </c>
-      <c r="J18" t="s">
-        <v>0</v>
-      </c>
-      <c r="K18" t="b">
-        <v>1</v>
-      </c>
-      <c r="L18" t="b">
-        <v>0</v>
-      </c>
-      <c r="M18" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>1.2</v>
-      </c>
-      <c r="O18">
-        <v>24</v>
-      </c>
-      <c r="P18" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1761,40 +1345,19 @@
       <c r="H19">
         <v>3</v>
       </c>
-      <c r="I19">
-        <v>3</v>
-      </c>
-      <c r="J19" t="s">
-        <v>0</v>
-      </c>
-      <c r="K19" t="b">
-        <v>1</v>
-      </c>
-      <c r="L19" t="b">
-        <v>0</v>
-      </c>
-      <c r="M19" t="b">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>1.3</v>
-      </c>
-      <c r="O19">
-        <v>26</v>
-      </c>
-      <c r="P19" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -1811,40 +1374,19 @@
       <c r="H20">
         <v>3</v>
       </c>
-      <c r="I20">
-        <v>3</v>
-      </c>
-      <c r="J20" t="s">
-        <v>0</v>
-      </c>
-      <c r="K20" t="b">
-        <v>1</v>
-      </c>
-      <c r="L20" t="b">
-        <v>0</v>
-      </c>
-      <c r="M20" t="b">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>1.5</v>
-      </c>
-      <c r="O20">
-        <v>28</v>
-      </c>
-      <c r="P20" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1861,40 +1403,19 @@
       <c r="H21">
         <v>1</v>
       </c>
-      <c r="I21">
-        <v>1</v>
-      </c>
-      <c r="J21" t="s">
-        <v>8</v>
-      </c>
-      <c r="K21" t="b">
-        <v>1</v>
-      </c>
-      <c r="L21" t="b">
-        <v>0</v>
-      </c>
-      <c r="M21" t="b">
-        <v>0</v>
-      </c>
-      <c r="N21">
-        <v>0.8</v>
-      </c>
-      <c r="O21">
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>18</v>
       </c>
-      <c r="P21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
       <c r="B22" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -1911,40 +1432,19 @@
       <c r="H22">
         <v>0.1</v>
       </c>
-      <c r="I22">
-        <v>1</v>
-      </c>
-      <c r="J22" t="s">
-        <v>4</v>
-      </c>
-      <c r="K22" t="b">
-        <v>0</v>
-      </c>
-      <c r="L22" t="b">
-        <v>0</v>
-      </c>
-      <c r="M22" t="b">
-        <v>0</v>
-      </c>
-      <c r="N22">
-        <v>0.2</v>
-      </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1961,40 +1461,19 @@
       <c r="H23">
         <v>0.2</v>
       </c>
-      <c r="I23">
-        <v>1</v>
-      </c>
-      <c r="J23" t="s">
-        <v>4</v>
-      </c>
-      <c r="K23" t="b">
-        <v>1</v>
-      </c>
-      <c r="L23" t="b">
-        <v>0</v>
-      </c>
-      <c r="M23" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23">
-        <v>0.4</v>
-      </c>
-      <c r="O23">
-        <v>0</v>
-      </c>
-      <c r="P23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -2011,40 +1490,19 @@
       <c r="H24">
         <v>0.5</v>
       </c>
-      <c r="I24">
-        <v>1</v>
-      </c>
-      <c r="J24" t="s">
-        <v>8</v>
-      </c>
-      <c r="K24" t="b">
-        <v>1</v>
-      </c>
-      <c r="L24" t="b">
+      <c r="I24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" t="s">
         <v>0</v>
-      </c>
-      <c r="M24" t="b">
-        <v>0</v>
-      </c>
-      <c r="N24">
-        <v>0.6</v>
-      </c>
-      <c r="O24">
-        <v>10</v>
-      </c>
-      <c r="P24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" t="s">
-        <v>1</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -2061,40 +1519,19 @@
       <c r="H25">
         <v>1.5</v>
       </c>
-      <c r="I25">
-        <v>2</v>
-      </c>
-      <c r="J25" t="s">
-        <v>0</v>
-      </c>
-      <c r="K25" t="b">
-        <v>1</v>
-      </c>
-      <c r="L25" t="b">
-        <v>0</v>
-      </c>
-      <c r="M25" t="b">
-        <v>1</v>
-      </c>
-      <c r="N25">
-        <v>1</v>
-      </c>
-      <c r="O25">
-        <v>22</v>
-      </c>
-      <c r="P25" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -2111,40 +1548,19 @@
       <c r="H26">
         <v>1.5</v>
       </c>
-      <c r="I26">
-        <v>2</v>
-      </c>
-      <c r="J26" t="s">
-        <v>8</v>
-      </c>
-      <c r="K26" t="b">
-        <v>1</v>
-      </c>
-      <c r="L26" t="b">
-        <v>0</v>
-      </c>
-      <c r="M26" t="b">
-        <v>0</v>
-      </c>
-      <c r="N26">
-        <v>1</v>
-      </c>
-      <c r="O26">
-        <v>18</v>
-      </c>
-      <c r="P26" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2161,40 +1577,19 @@
       <c r="H27">
         <v>2.5</v>
       </c>
-      <c r="I27">
-        <v>2</v>
-      </c>
-      <c r="J27" t="s">
-        <v>0</v>
-      </c>
-      <c r="K27" t="b">
-        <v>1</v>
-      </c>
-      <c r="L27" t="b">
-        <v>0</v>
-      </c>
-      <c r="M27" t="b">
-        <v>0</v>
-      </c>
-      <c r="N27">
-        <v>1.3</v>
-      </c>
-      <c r="O27">
-        <v>28</v>
-      </c>
-      <c r="P27" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D28">
         <v>2</v>
@@ -2211,40 +1606,19 @@
       <c r="H28">
         <v>3</v>
       </c>
-      <c r="I28">
-        <v>3</v>
-      </c>
-      <c r="J28" t="s">
-        <v>0</v>
-      </c>
-      <c r="K28" t="b">
-        <v>1</v>
-      </c>
-      <c r="L28" t="b">
-        <v>0</v>
-      </c>
-      <c r="M28" t="b">
-        <v>0</v>
-      </c>
-      <c r="N28">
-        <v>1.5</v>
-      </c>
-      <c r="O28">
-        <v>32</v>
-      </c>
-      <c r="P28" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B29" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D29">
         <v>2</v>
@@ -2261,40 +1635,19 @@
       <c r="H29">
         <v>1</v>
       </c>
-      <c r="I29">
-        <v>1</v>
-      </c>
-      <c r="J29" t="s">
-        <v>0</v>
-      </c>
-      <c r="K29" t="b">
-        <v>1</v>
-      </c>
-      <c r="L29" t="b">
-        <v>0</v>
-      </c>
-      <c r="M29" t="b">
-        <v>0</v>
-      </c>
-      <c r="N29">
-        <v>0.8</v>
-      </c>
-      <c r="O29">
-        <v>10</v>
-      </c>
-      <c r="P29" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D30">
         <v>3</v>
@@ -2311,40 +1664,19 @@
       <c r="H30">
         <v>0.8</v>
       </c>
-      <c r="I30">
-        <v>1</v>
-      </c>
-      <c r="J30" t="s">
-        <v>8</v>
-      </c>
-      <c r="K30" t="b">
-        <v>1</v>
-      </c>
-      <c r="L30" t="b">
-        <v>0</v>
-      </c>
-      <c r="M30" t="b">
-        <v>0</v>
-      </c>
-      <c r="N30">
-        <v>0.7</v>
-      </c>
-      <c r="O30">
-        <v>14</v>
-      </c>
-      <c r="P30" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -2361,40 +1693,19 @@
       <c r="H31">
         <v>0.2</v>
       </c>
-      <c r="I31">
-        <v>1</v>
-      </c>
-      <c r="J31" t="s">
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>4</v>
       </c>
-      <c r="K31" t="b">
-        <v>1</v>
-      </c>
-      <c r="L31" t="b">
-        <v>0</v>
-      </c>
-      <c r="M31" t="b">
-        <v>0</v>
-      </c>
-      <c r="N31">
-        <v>0.4</v>
-      </c>
-      <c r="O31">
-        <v>0</v>
-      </c>
-      <c r="P31" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>6</v>
-      </c>
       <c r="B32" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -2411,40 +1722,19 @@
       <c r="H32">
         <v>0.3</v>
       </c>
-      <c r="I32">
-        <v>1</v>
-      </c>
-      <c r="J32" t="s">
-        <v>4</v>
-      </c>
-      <c r="K32" t="b">
-        <v>1</v>
-      </c>
-      <c r="L32" t="b">
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
         <v>0</v>
-      </c>
-      <c r="M32" t="b">
-        <v>0</v>
-      </c>
-      <c r="N32">
-        <v>0.8</v>
-      </c>
-      <c r="O32">
-        <v>0</v>
-      </c>
-      <c r="P32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" t="s">
-        <v>2</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1</v>
       </c>
       <c r="D33">
         <v>4</v>
@@ -2461,28 +1751,7 @@
       <c r="H33">
         <v>2</v>
       </c>
-      <c r="I33">
-        <v>3</v>
-      </c>
-      <c r="J33" t="s">
-        <v>0</v>
-      </c>
-      <c r="K33" t="b">
-        <v>1</v>
-      </c>
-      <c r="L33" t="b">
-        <v>0</v>
-      </c>
-      <c r="M33" t="b">
-        <v>1</v>
-      </c>
-      <c r="N33">
-        <v>1.5</v>
-      </c>
-      <c r="O33">
-        <v>45</v>
-      </c>
-      <c r="P33" t="b">
+      <c r="I33" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2507,24 +1776,24 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" t="s">
         <v>59</v>
-      </c>
-      <c r="B1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C2">
         <v>0.75</v>
@@ -2535,10 +1804,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C3">
         <v>0.8</v>
@@ -2549,10 +1818,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C4">
         <v>0.18</v>
@@ -2563,10 +1832,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C5">
         <v>0.7</v>
@@ -2577,10 +1846,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C6">
         <v>0.65</v>
@@ -2591,10 +1860,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C7">
         <v>0.22</v>
@@ -2605,10 +1874,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <v>0.75</v>
@@ -2619,10 +1888,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C9">
         <v>0.45</v>
@@ -2633,10 +1902,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C10">
         <v>0.35</v>
@@ -2647,10 +1916,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C11">
         <v>0.55000000000000004</v>
@@ -2661,10 +1930,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C12">
         <v>0.3</v>
@@ -2675,10 +1944,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C13">
         <v>0.12</v>
@@ -2689,10 +1958,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C14">
         <v>0.55000000000000004</v>
@@ -2703,10 +1972,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C15">
         <v>0.65</v>
@@ -2717,10 +1986,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C16">
         <v>0.4</v>
@@ -2731,10 +2000,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C17">
         <v>0.6</v>
@@ -2745,10 +2014,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C18">
         <v>0.38</v>
@@ -2778,21 +2047,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2806,7 +2075,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B3">
         <v>0.35</v>
@@ -2820,7 +2089,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B4">
         <v>-0.7</v>
@@ -2852,18 +2121,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2874,7 +2143,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B3">
         <v>0.25</v>
@@ -2906,30 +2175,30 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="F1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2952,7 +2221,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B3">
         <v>-0.6</v>
@@ -2975,7 +2244,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B4">
         <v>-0.55000000000000004</v>
@@ -2998,7 +2267,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B5">
         <v>-0.35</v>
@@ -3021,7 +2290,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B6">
         <v>-0.25</v>
@@ -3044,7 +2313,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B7">
         <v>-0.2</v>
@@ -3089,30 +2358,30 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="F1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -3135,7 +2404,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B3">
         <v>-0.55000000000000004</v>
@@ -3158,7 +2427,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B4">
         <v>-0.6</v>
@@ -3181,7 +2450,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B5">
         <v>-0.3</v>
@@ -3204,7 +2473,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B6">
         <v>-0.2</v>
@@ -3227,7 +2496,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B7">
         <v>-0.15</v>

</xml_diff>